<commit_message>
First upload of forecast notebook
</commit_message>
<xml_diff>
--- a/SquareSalesProcessingAndForecast/pivot_plus_forecast.xlsx
+++ b/SquareSalesProcessingAndForecast/pivot_plus_forecast.xlsx
@@ -28847,19 +28847,19 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
+          <t>Grilled zucchinis</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Water</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
           <t>Tofu cutlet</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>Grilled zucchinis</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>Water</t>
-        </is>
-      </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Chicken thighs</t>
@@ -28912,12 +28912,12 @@
       </c>
       <c r="T1" s="1" t="inlineStr">
         <is>
+          <t>Chicken skin</t>
+        </is>
+      </c>
+      <c r="U1" s="1" t="inlineStr">
+        <is>
           <t>Ice green tea</t>
-        </is>
-      </c>
-      <c r="U1" s="1" t="inlineStr">
-        <is>
-          <t>Chicken skin</t>
         </is>
       </c>
       <c r="V1" s="1" t="inlineStr">
@@ -29017,13 +29017,13 @@
         <v>10</v>
       </c>
       <c r="G2" t="n">
+        <v>3</v>
+      </c>
+      <c r="H2" t="n">
+        <v>8</v>
+      </c>
+      <c r="I2" t="n">
         <v>11</v>
-      </c>
-      <c r="H2" t="n">
-        <v>3</v>
-      </c>
-      <c r="I2" t="n">
-        <v>8</v>
       </c>
       <c r="J2" t="n">
         <v>34</v>
@@ -29056,10 +29056,10 @@
         <v>2</v>
       </c>
       <c r="T2" t="n">
+        <v>1</v>
+      </c>
+      <c r="U2" t="n">
         <v>4</v>
-      </c>
-      <c r="U2" t="n">
-        <v>1</v>
       </c>
       <c r="V2" t="n">
         <v>1</v>
@@ -29356,13 +29356,13 @@
         <v>3</v>
       </c>
       <c r="G5" t="n">
+        <v>2</v>
+      </c>
+      <c r="H5" t="n">
+        <v>6</v>
+      </c>
+      <c r="I5" t="n">
         <v>8</v>
-      </c>
-      <c r="H5" t="n">
-        <v>2</v>
-      </c>
-      <c r="I5" t="n">
-        <v>6</v>
       </c>
       <c r="J5" t="n">
         <v>20</v>
@@ -29695,13 +29695,13 @@
         <v>11</v>
       </c>
       <c r="G8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" t="n">
+        <v>4</v>
+      </c>
+      <c r="I8" t="n">
         <v>13</v>
-      </c>
-      <c r="H8" t="n">
-        <v>0</v>
-      </c>
-      <c r="I8" t="n">
-        <v>4</v>
       </c>
       <c r="J8" t="n">
         <v>20</v>
@@ -29734,10 +29734,10 @@
         <v>0</v>
       </c>
       <c r="T8" t="n">
+        <v>2</v>
+      </c>
+      <c r="U8" t="n">
         <v>5</v>
-      </c>
-      <c r="U8" t="n">
-        <v>2</v>
       </c>
       <c r="V8" t="n">
         <v>0</v>
@@ -30034,13 +30034,13 @@
         <v>7</v>
       </c>
       <c r="G11" t="n">
+        <v>1</v>
+      </c>
+      <c r="H11" t="n">
+        <v>6</v>
+      </c>
+      <c r="I11" t="n">
         <v>9</v>
-      </c>
-      <c r="H11" t="n">
-        <v>1</v>
-      </c>
-      <c r="I11" t="n">
-        <v>6</v>
       </c>
       <c r="J11" t="n">
         <v>8</v>
@@ -30073,10 +30073,10 @@
         <v>4</v>
       </c>
       <c r="T11" t="n">
+        <v>0</v>
+      </c>
+      <c r="U11" t="n">
         <v>2</v>
-      </c>
-      <c r="U11" t="n">
-        <v>0</v>
       </c>
       <c r="V11" t="n">
         <v>0</v>
@@ -30373,13 +30373,13 @@
         <v>6</v>
       </c>
       <c r="G14" t="n">
+        <v>2</v>
+      </c>
+      <c r="H14" t="n">
+        <v>1</v>
+      </c>
+      <c r="I14" t="n">
         <v>6</v>
-      </c>
-      <c r="H14" t="n">
-        <v>2</v>
-      </c>
-      <c r="I14" t="n">
-        <v>1</v>
       </c>
       <c r="J14" t="n">
         <v>13</v>
@@ -30412,10 +30412,10 @@
         <v>2</v>
       </c>
       <c r="T14" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="U14" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="V14" t="n">
         <v>0</v>
@@ -30712,13 +30712,13 @@
         <v>11</v>
       </c>
       <c r="G17" t="n">
+        <v>5</v>
+      </c>
+      <c r="H17" t="n">
+        <v>16</v>
+      </c>
+      <c r="I17" t="n">
         <v>21</v>
-      </c>
-      <c r="H17" t="n">
-        <v>5</v>
-      </c>
-      <c r="I17" t="n">
-        <v>16</v>
       </c>
       <c r="J17" t="n">
         <v>34</v>
@@ -30751,10 +30751,10 @@
         <v>6</v>
       </c>
       <c r="T17" t="n">
+        <v>1</v>
+      </c>
+      <c r="U17" t="n">
         <v>4</v>
-      </c>
-      <c r="U17" t="n">
-        <v>1</v>
       </c>
       <c r="V17" t="n">
         <v>0</v>
@@ -31051,13 +31051,13 @@
         <v>11</v>
       </c>
       <c r="G20" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="H20" t="n">
         <v>1</v>
       </c>
       <c r="I20" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="J20" t="n">
         <v>12</v>
@@ -31390,13 +31390,13 @@
         <v>9</v>
       </c>
       <c r="G23" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="H23" t="n">
         <v>1</v>
       </c>
       <c r="I23" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="J23" t="n">
         <v>24</v>
@@ -31429,10 +31429,10 @@
         <v>2</v>
       </c>
       <c r="T23" t="n">
+        <v>2</v>
+      </c>
+      <c r="U23" t="n">
         <v>4</v>
-      </c>
-      <c r="U23" t="n">
-        <v>2</v>
       </c>
       <c r="V23" t="n">
         <v>0</v>
@@ -31729,13 +31729,13 @@
         <v>5</v>
       </c>
       <c r="G26" t="n">
+        <v>0</v>
+      </c>
+      <c r="H26" t="n">
+        <v>3</v>
+      </c>
+      <c r="I26" t="n">
         <v>7</v>
-      </c>
-      <c r="H26" t="n">
-        <v>0</v>
-      </c>
-      <c r="I26" t="n">
-        <v>3</v>
       </c>
       <c r="J26" t="n">
         <v>18</v>
@@ -32068,13 +32068,13 @@
         <v>7</v>
       </c>
       <c r="G29" t="n">
+        <v>2</v>
+      </c>
+      <c r="H29" t="n">
+        <v>7</v>
+      </c>
+      <c r="I29" t="n">
         <v>10</v>
-      </c>
-      <c r="H29" t="n">
-        <v>2</v>
-      </c>
-      <c r="I29" t="n">
-        <v>7</v>
       </c>
       <c r="J29" t="n">
         <v>10</v>
@@ -32107,10 +32107,10 @@
         <v>2</v>
       </c>
       <c r="T29" t="n">
+        <v>1</v>
+      </c>
+      <c r="U29" t="n">
         <v>2</v>
-      </c>
-      <c r="U29" t="n">
-        <v>1</v>
       </c>
       <c r="V29" t="n">
         <v>1</v>
@@ -32407,13 +32407,13 @@
         <v>8</v>
       </c>
       <c r="G32" t="n">
+        <v>5</v>
+      </c>
+      <c r="H32" t="n">
+        <v>9</v>
+      </c>
+      <c r="I32" t="n">
         <v>10</v>
-      </c>
-      <c r="H32" t="n">
-        <v>5</v>
-      </c>
-      <c r="I32" t="n">
-        <v>9</v>
       </c>
       <c r="J32" t="n">
         <v>38</v>
@@ -32446,10 +32446,10 @@
         <v>5</v>
       </c>
       <c r="T32" t="n">
+        <v>2</v>
+      </c>
+      <c r="U32" t="n">
         <v>3</v>
-      </c>
-      <c r="U32" t="n">
-        <v>2</v>
       </c>
       <c r="V32" t="n">
         <v>0</v>
@@ -32746,13 +32746,13 @@
         <v>15</v>
       </c>
       <c r="G35" t="n">
+        <v>3</v>
+      </c>
+      <c r="H35" t="n">
+        <v>6</v>
+      </c>
+      <c r="I35" t="n">
         <v>13</v>
-      </c>
-      <c r="H35" t="n">
-        <v>3</v>
-      </c>
-      <c r="I35" t="n">
-        <v>6</v>
       </c>
       <c r="J35" t="n">
         <v>38</v>
@@ -32785,10 +32785,10 @@
         <v>5</v>
       </c>
       <c r="T35" t="n">
+        <v>1</v>
+      </c>
+      <c r="U35" t="n">
         <v>4</v>
-      </c>
-      <c r="U35" t="n">
-        <v>1</v>
       </c>
       <c r="V35" t="n">
         <v>2</v>
@@ -33085,13 +33085,13 @@
         <v>16</v>
       </c>
       <c r="G38" t="n">
+        <v>8</v>
+      </c>
+      <c r="H38" t="n">
+        <v>19</v>
+      </c>
+      <c r="I38" t="n">
         <v>22</v>
-      </c>
-      <c r="H38" t="n">
-        <v>8</v>
-      </c>
-      <c r="I38" t="n">
-        <v>19</v>
       </c>
       <c r="J38" t="n">
         <v>66</v>
@@ -33124,10 +33124,10 @@
         <v>9</v>
       </c>
       <c r="T38" t="n">
+        <v>0</v>
+      </c>
+      <c r="U38" t="n">
         <v>1</v>
-      </c>
-      <c r="U38" t="n">
-        <v>0</v>
       </c>
       <c r="V38" t="n">
         <v>1</v>
@@ -33424,13 +33424,13 @@
         <v>9</v>
       </c>
       <c r="G41" t="n">
+        <v>2</v>
+      </c>
+      <c r="H41" t="n">
+        <v>8</v>
+      </c>
+      <c r="I41" t="n">
         <v>16</v>
-      </c>
-      <c r="H41" t="n">
-        <v>2</v>
-      </c>
-      <c r="I41" t="n">
-        <v>8</v>
       </c>
       <c r="J41" t="n">
         <v>20</v>
@@ -33763,10 +33763,10 @@
         <v>3</v>
       </c>
       <c r="G44" t="n">
+        <v>1</v>
+      </c>
+      <c r="H44" t="n">
         <v>5</v>
-      </c>
-      <c r="H44" t="n">
-        <v>1</v>
       </c>
       <c r="I44" t="n">
         <v>5</v>
@@ -34102,13 +34102,13 @@
         <v>9</v>
       </c>
       <c r="G47" t="n">
+        <v>1</v>
+      </c>
+      <c r="H47" t="n">
+        <v>3</v>
+      </c>
+      <c r="I47" t="n">
         <v>8</v>
-      </c>
-      <c r="H47" t="n">
-        <v>1</v>
-      </c>
-      <c r="I47" t="n">
-        <v>3</v>
       </c>
       <c r="J47" t="n">
         <v>13</v>
@@ -34441,13 +34441,13 @@
         <v>7</v>
       </c>
       <c r="G50" t="n">
+        <v>0</v>
+      </c>
+      <c r="H50" t="n">
+        <v>4</v>
+      </c>
+      <c r="I50" t="n">
         <v>6</v>
-      </c>
-      <c r="H50" t="n">
-        <v>0</v>
-      </c>
-      <c r="I50" t="n">
-        <v>4</v>
       </c>
       <c r="J50" t="n">
         <v>14</v>
@@ -34480,10 +34480,10 @@
         <v>5</v>
       </c>
       <c r="T50" t="n">
+        <v>0</v>
+      </c>
+      <c r="U50" t="n">
         <v>2</v>
-      </c>
-      <c r="U50" t="n">
-        <v>0</v>
       </c>
       <c r="V50" t="n">
         <v>0</v>
@@ -34780,13 +34780,13 @@
         <v>9</v>
       </c>
       <c r="G53" t="n">
+        <v>0</v>
+      </c>
+      <c r="H53" t="n">
+        <v>3</v>
+      </c>
+      <c r="I53" t="n">
         <v>7</v>
-      </c>
-      <c r="H53" t="n">
-        <v>0</v>
-      </c>
-      <c r="I53" t="n">
-        <v>3</v>
       </c>
       <c r="J53" t="n">
         <v>30</v>
@@ -34819,10 +34819,10 @@
         <v>1</v>
       </c>
       <c r="T53" t="n">
+        <v>0</v>
+      </c>
+      <c r="U53" t="n">
         <v>4</v>
-      </c>
-      <c r="U53" t="n">
-        <v>0</v>
       </c>
       <c r="V53" t="n">
         <v>0</v>
@@ -35119,13 +35119,13 @@
         <v>9</v>
       </c>
       <c r="G56" t="n">
+        <v>2</v>
+      </c>
+      <c r="H56" t="n">
+        <v>1</v>
+      </c>
+      <c r="I56" t="n">
         <v>7</v>
-      </c>
-      <c r="H56" t="n">
-        <v>2</v>
-      </c>
-      <c r="I56" t="n">
-        <v>1</v>
       </c>
       <c r="J56" t="n">
         <v>16</v>
@@ -35158,10 +35158,10 @@
         <v>2</v>
       </c>
       <c r="T56" t="n">
+        <v>0</v>
+      </c>
+      <c r="U56" t="n">
         <v>2</v>
-      </c>
-      <c r="U56" t="n">
-        <v>0</v>
       </c>
       <c r="V56" t="n">
         <v>0</v>
@@ -35458,13 +35458,13 @@
         <v>15</v>
       </c>
       <c r="G59" t="n">
+        <v>1</v>
+      </c>
+      <c r="H59" t="n">
+        <v>12</v>
+      </c>
+      <c r="I59" t="n">
         <v>11</v>
-      </c>
-      <c r="H59" t="n">
-        <v>1</v>
-      </c>
-      <c r="I59" t="n">
-        <v>12</v>
       </c>
       <c r="J59" t="n">
         <v>36</v>
@@ -35497,10 +35497,10 @@
         <v>7</v>
       </c>
       <c r="T59" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U59" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="V59" t="n">
         <v>0</v>
@@ -35797,13 +35797,13 @@
         <v>11</v>
       </c>
       <c r="G62" t="n">
+        <v>0</v>
+      </c>
+      <c r="H62" t="n">
+        <v>5</v>
+      </c>
+      <c r="I62" t="n">
         <v>9</v>
-      </c>
-      <c r="H62" t="n">
-        <v>0</v>
-      </c>
-      <c r="I62" t="n">
-        <v>5</v>
       </c>
       <c r="J62" t="n">
         <v>17</v>
@@ -35836,10 +35836,10 @@
         <v>0</v>
       </c>
       <c r="T62" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U62" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="V62" t="n">
         <v>0</v>
@@ -36136,13 +36136,13 @@
         <v>6</v>
       </c>
       <c r="G65" t="n">
+        <v>2</v>
+      </c>
+      <c r="H65" t="n">
+        <v>3</v>
+      </c>
+      <c r="I65" t="n">
         <v>8</v>
-      </c>
-      <c r="H65" t="n">
-        <v>2</v>
-      </c>
-      <c r="I65" t="n">
-        <v>3</v>
       </c>
       <c r="J65" t="n">
         <v>11</v>
@@ -36175,10 +36175,10 @@
         <v>3</v>
       </c>
       <c r="T65" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U65" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="V65" t="n">
         <v>0</v>
@@ -36475,13 +36475,13 @@
         <v>5</v>
       </c>
       <c r="G68" t="n">
+        <v>2</v>
+      </c>
+      <c r="H68" t="n">
+        <v>7</v>
+      </c>
+      <c r="I68" t="n">
         <v>14</v>
-      </c>
-      <c r="H68" t="n">
-        <v>2</v>
-      </c>
-      <c r="I68" t="n">
-        <v>7</v>
       </c>
       <c r="J68" t="n">
         <v>16</v>
@@ -36514,10 +36514,10 @@
         <v>2</v>
       </c>
       <c r="T68" t="n">
+        <v>0</v>
+      </c>
+      <c r="U68" t="n">
         <v>3</v>
-      </c>
-      <c r="U68" t="n">
-        <v>0</v>
       </c>
       <c r="V68" t="n">
         <v>0</v>
@@ -36814,13 +36814,13 @@
         <v>3</v>
       </c>
       <c r="G71" t="n">
+        <v>0</v>
+      </c>
+      <c r="H71" t="n">
+        <v>4</v>
+      </c>
+      <c r="I71" t="n">
         <v>9</v>
-      </c>
-      <c r="H71" t="n">
-        <v>0</v>
-      </c>
-      <c r="I71" t="n">
-        <v>4</v>
       </c>
       <c r="J71" t="n">
         <v>17</v>
@@ -36853,10 +36853,10 @@
         <v>3</v>
       </c>
       <c r="T71" t="n">
+        <v>0</v>
+      </c>
+      <c r="U71" t="n">
         <v>2</v>
-      </c>
-      <c r="U71" t="n">
-        <v>0</v>
       </c>
       <c r="V71" t="n">
         <v>0</v>
@@ -37153,13 +37153,13 @@
         <v>20</v>
       </c>
       <c r="G74" t="n">
+        <v>4</v>
+      </c>
+      <c r="H74" t="n">
+        <v>5</v>
+      </c>
+      <c r="I74" t="n">
         <v>12</v>
-      </c>
-      <c r="H74" t="n">
-        <v>4</v>
-      </c>
-      <c r="I74" t="n">
-        <v>5</v>
       </c>
       <c r="J74" t="n">
         <v>9</v>
@@ -37492,13 +37492,13 @@
         <v>4</v>
       </c>
       <c r="G77" t="n">
+        <v>0</v>
+      </c>
+      <c r="H77" t="n">
+        <v>3</v>
+      </c>
+      <c r="I77" t="n">
         <v>17</v>
-      </c>
-      <c r="H77" t="n">
-        <v>0</v>
-      </c>
-      <c r="I77" t="n">
-        <v>3</v>
       </c>
       <c r="J77" t="n">
         <v>24</v>
@@ -37531,10 +37531,10 @@
         <v>4</v>
       </c>
       <c r="T77" t="n">
+        <v>0</v>
+      </c>
+      <c r="U77" t="n">
         <v>2</v>
-      </c>
-      <c r="U77" t="n">
-        <v>0</v>
       </c>
       <c r="V77" t="n">
         <v>1</v>
@@ -37831,13 +37831,13 @@
         <v>9</v>
       </c>
       <c r="G80" t="n">
+        <v>1</v>
+      </c>
+      <c r="H80" t="n">
+        <v>9</v>
+      </c>
+      <c r="I80" t="n">
         <v>14</v>
-      </c>
-      <c r="H80" t="n">
-        <v>1</v>
-      </c>
-      <c r="I80" t="n">
-        <v>9</v>
       </c>
       <c r="J80" t="n">
         <v>41</v>
@@ -38170,10 +38170,10 @@
         <v>11</v>
       </c>
       <c r="G83" t="n">
+        <v>0</v>
+      </c>
+      <c r="H83" t="n">
         <v>11</v>
-      </c>
-      <c r="H83" t="n">
-        <v>0</v>
       </c>
       <c r="I83" t="n">
         <v>11</v>
@@ -38209,10 +38209,10 @@
         <v>3</v>
       </c>
       <c r="T83" t="n">
+        <v>0</v>
+      </c>
+      <c r="U83" t="n">
         <v>1</v>
-      </c>
-      <c r="U83" t="n">
-        <v>0</v>
       </c>
       <c r="V83" t="n">
         <v>0</v>
@@ -38509,13 +38509,13 @@
         <v>16</v>
       </c>
       <c r="G86" t="n">
+        <v>2</v>
+      </c>
+      <c r="H86" t="n">
+        <v>8</v>
+      </c>
+      <c r="I86" t="n">
         <v>17</v>
-      </c>
-      <c r="H86" t="n">
-        <v>2</v>
-      </c>
-      <c r="I86" t="n">
-        <v>8</v>
       </c>
       <c r="J86" t="n">
         <v>34</v>
@@ -38548,10 +38548,10 @@
         <v>4</v>
       </c>
       <c r="T86" t="n">
+        <v>1</v>
+      </c>
+      <c r="U86" t="n">
         <v>4</v>
-      </c>
-      <c r="U86" t="n">
-        <v>1</v>
       </c>
       <c r="V86" t="n">
         <v>0</v>
@@ -38848,13 +38848,13 @@
         <v>5</v>
       </c>
       <c r="G89" t="n">
+        <v>3</v>
+      </c>
+      <c r="H89" t="n">
+        <v>7</v>
+      </c>
+      <c r="I89" t="n">
         <v>17</v>
-      </c>
-      <c r="H89" t="n">
-        <v>3</v>
-      </c>
-      <c r="I89" t="n">
-        <v>7</v>
       </c>
       <c r="J89" t="n">
         <v>9</v>
@@ -38887,10 +38887,10 @@
         <v>5</v>
       </c>
       <c r="T89" t="n">
+        <v>0</v>
+      </c>
+      <c r="U89" t="n">
         <v>3</v>
-      </c>
-      <c r="U89" t="n">
-        <v>0</v>
       </c>
       <c r="V89" t="n">
         <v>0</v>
@@ -39187,13 +39187,13 @@
         <v>9</v>
       </c>
       <c r="G92" t="n">
+        <v>2</v>
+      </c>
+      <c r="H92" t="n">
+        <v>10</v>
+      </c>
+      <c r="I92" t="n">
         <v>15</v>
-      </c>
-      <c r="H92" t="n">
-        <v>2</v>
-      </c>
-      <c r="I92" t="n">
-        <v>10</v>
       </c>
       <c r="J92" t="n">
         <v>13</v>
@@ -39226,10 +39226,10 @@
         <v>0</v>
       </c>
       <c r="T92" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="U92" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="V92" t="n">
         <v>1</v>
@@ -39526,13 +39526,13 @@
         <v>10</v>
       </c>
       <c r="G95" t="n">
+        <v>1</v>
+      </c>
+      <c r="H95" t="n">
+        <v>5</v>
+      </c>
+      <c r="I95" t="n">
         <v>6</v>
-      </c>
-      <c r="H95" t="n">
-        <v>1</v>
-      </c>
-      <c r="I95" t="n">
-        <v>5</v>
       </c>
       <c r="J95" t="n">
         <v>17</v>
@@ -39565,10 +39565,10 @@
         <v>4</v>
       </c>
       <c r="T95" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U95" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="V95" t="n">
         <v>0</v>
@@ -39865,13 +39865,13 @@
         <v>12</v>
       </c>
       <c r="G98" t="n">
+        <v>1</v>
+      </c>
+      <c r="H98" t="n">
+        <v>5</v>
+      </c>
+      <c r="I98" t="n">
         <v>7</v>
-      </c>
-      <c r="H98" t="n">
-        <v>1</v>
-      </c>
-      <c r="I98" t="n">
-        <v>5</v>
       </c>
       <c r="J98" t="n">
         <v>13</v>
@@ -40204,13 +40204,13 @@
         <v>6</v>
       </c>
       <c r="G101" t="n">
+        <v>1</v>
+      </c>
+      <c r="H101" t="n">
+        <v>4</v>
+      </c>
+      <c r="I101" t="n">
         <v>15</v>
-      </c>
-      <c r="H101" t="n">
-        <v>1</v>
-      </c>
-      <c r="I101" t="n">
-        <v>4</v>
       </c>
       <c r="J101" t="n">
         <v>22</v>
@@ -40243,10 +40243,10 @@
         <v>3</v>
       </c>
       <c r="T101" t="n">
+        <v>0</v>
+      </c>
+      <c r="U101" t="n">
         <v>2</v>
-      </c>
-      <c r="U101" t="n">
-        <v>0</v>
       </c>
       <c r="V101" t="n">
         <v>0</v>
@@ -40543,13 +40543,13 @@
         <v>11</v>
       </c>
       <c r="G104" t="n">
+        <v>3</v>
+      </c>
+      <c r="H104" t="n">
+        <v>10</v>
+      </c>
+      <c r="I104" t="n">
         <v>15</v>
-      </c>
-      <c r="H104" t="n">
-        <v>3</v>
-      </c>
-      <c r="I104" t="n">
-        <v>10</v>
       </c>
       <c r="J104" t="n">
         <v>25</v>
@@ -40582,10 +40582,10 @@
         <v>5</v>
       </c>
       <c r="T104" t="n">
+        <v>1</v>
+      </c>
+      <c r="U104" t="n">
         <v>7</v>
-      </c>
-      <c r="U104" t="n">
-        <v>1</v>
       </c>
       <c r="V104" t="n">
         <v>0</v>
@@ -40882,13 +40882,13 @@
         <v>3</v>
       </c>
       <c r="G107" t="n">
+        <v>2</v>
+      </c>
+      <c r="H107" t="n">
+        <v>7</v>
+      </c>
+      <c r="I107" t="n">
         <v>8</v>
-      </c>
-      <c r="H107" t="n">
-        <v>2</v>
-      </c>
-      <c r="I107" t="n">
-        <v>7</v>
       </c>
       <c r="J107" t="n">
         <v>15</v>
@@ -40921,10 +40921,10 @@
         <v>2</v>
       </c>
       <c r="T107" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U107" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="V107" t="n">
         <v>0</v>
@@ -41221,13 +41221,13 @@
         <v>10</v>
       </c>
       <c r="G110" t="n">
+        <v>2</v>
+      </c>
+      <c r="H110" t="n">
+        <v>6</v>
+      </c>
+      <c r="I110" t="n">
         <v>9</v>
-      </c>
-      <c r="H110" t="n">
-        <v>2</v>
-      </c>
-      <c r="I110" t="n">
-        <v>6</v>
       </c>
       <c r="J110" t="n">
         <v>20</v>
@@ -41260,10 +41260,10 @@
         <v>3</v>
       </c>
       <c r="T110" t="n">
+        <v>0</v>
+      </c>
+      <c r="U110" t="n">
         <v>3</v>
-      </c>
-      <c r="U110" t="n">
-        <v>0</v>
       </c>
       <c r="V110" t="n">
         <v>1</v>
@@ -41560,13 +41560,13 @@
         <v>7</v>
       </c>
       <c r="G113" t="n">
+        <v>2</v>
+      </c>
+      <c r="H113" t="n">
+        <v>5</v>
+      </c>
+      <c r="I113" t="n">
         <v>9</v>
-      </c>
-      <c r="H113" t="n">
-        <v>2</v>
-      </c>
-      <c r="I113" t="n">
-        <v>5</v>
       </c>
       <c r="J113" t="n">
         <v>23</v>
@@ -41599,10 +41599,10 @@
         <v>2</v>
       </c>
       <c r="T113" t="n">
+        <v>0</v>
+      </c>
+      <c r="U113" t="n">
         <v>1</v>
-      </c>
-      <c r="U113" t="n">
-        <v>0</v>
       </c>
       <c r="V113" t="n">
         <v>0</v>
@@ -41899,13 +41899,13 @@
         <v>12</v>
       </c>
       <c r="G116" t="n">
+        <v>1</v>
+      </c>
+      <c r="H116" t="n">
+        <v>12</v>
+      </c>
+      <c r="I116" t="n">
         <v>14</v>
-      </c>
-      <c r="H116" t="n">
-        <v>1</v>
-      </c>
-      <c r="I116" t="n">
-        <v>12</v>
       </c>
       <c r="J116" t="n">
         <v>20</v>
@@ -41938,10 +41938,10 @@
         <v>5</v>
       </c>
       <c r="T116" t="n">
+        <v>1</v>
+      </c>
+      <c r="U116" t="n">
         <v>6</v>
-      </c>
-      <c r="U116" t="n">
-        <v>1</v>
       </c>
       <c r="V116" t="n">
         <v>0</v>
@@ -42238,13 +42238,13 @@
         <v>5</v>
       </c>
       <c r="G119" t="n">
+        <v>3</v>
+      </c>
+      <c r="H119" t="n">
+        <v>4</v>
+      </c>
+      <c r="I119" t="n">
         <v>9</v>
-      </c>
-      <c r="H119" t="n">
-        <v>3</v>
-      </c>
-      <c r="I119" t="n">
-        <v>4</v>
       </c>
       <c r="J119" t="n">
         <v>23</v>
@@ -42577,10 +42577,10 @@
         <v>16</v>
       </c>
       <c r="G122" t="n">
+        <v>2</v>
+      </c>
+      <c r="H122" t="n">
         <v>11</v>
-      </c>
-      <c r="H122" t="n">
-        <v>2</v>
       </c>
       <c r="I122" t="n">
         <v>11</v>
@@ -42616,10 +42616,10 @@
         <v>5</v>
       </c>
       <c r="T122" t="n">
+        <v>2</v>
+      </c>
+      <c r="U122" t="n">
         <v>4</v>
-      </c>
-      <c r="U122" t="n">
-        <v>2</v>
       </c>
       <c r="V122" t="n">
         <v>0</v>
@@ -42916,13 +42916,13 @@
         <v>9</v>
       </c>
       <c r="G125" t="n">
+        <v>2</v>
+      </c>
+      <c r="H125" t="n">
+        <v>3</v>
+      </c>
+      <c r="I125" t="n">
         <v>6</v>
-      </c>
-      <c r="H125" t="n">
-        <v>2</v>
-      </c>
-      <c r="I125" t="n">
-        <v>3</v>
       </c>
       <c r="J125" t="n">
         <v>13</v>
@@ -43255,13 +43255,13 @@
         <v>5</v>
       </c>
       <c r="G128" t="n">
+        <v>0</v>
+      </c>
+      <c r="H128" t="n">
+        <v>7</v>
+      </c>
+      <c r="I128" t="n">
         <v>4</v>
-      </c>
-      <c r="H128" t="n">
-        <v>0</v>
-      </c>
-      <c r="I128" t="n">
-        <v>7</v>
       </c>
       <c r="J128" t="n">
         <v>22</v>
@@ -43294,10 +43294,10 @@
         <v>3</v>
       </c>
       <c r="T128" t="n">
+        <v>1</v>
+      </c>
+      <c r="U128" t="n">
         <v>2</v>
-      </c>
-      <c r="U128" t="n">
-        <v>1</v>
       </c>
       <c r="V128" t="n">
         <v>0</v>
@@ -43594,13 +43594,13 @@
         <v>5</v>
       </c>
       <c r="G131" t="n">
+        <v>0</v>
+      </c>
+      <c r="H131" t="n">
+        <v>4</v>
+      </c>
+      <c r="I131" t="n">
         <v>11</v>
-      </c>
-      <c r="H131" t="n">
-        <v>0</v>
-      </c>
-      <c r="I131" t="n">
-        <v>4</v>
       </c>
       <c r="J131" t="n">
         <v>10</v>
@@ -43633,10 +43633,10 @@
         <v>1</v>
       </c>
       <c r="T131" t="n">
+        <v>0</v>
+      </c>
+      <c r="U131" t="n">
         <v>4</v>
-      </c>
-      <c r="U131" t="n">
-        <v>0</v>
       </c>
       <c r="V131" t="n">
         <v>1</v>
@@ -43933,13 +43933,13 @@
         <v>8</v>
       </c>
       <c r="G134" t="n">
-        <v>14</v>
+        <v>2</v>
       </c>
       <c r="H134" t="n">
         <v>2</v>
       </c>
       <c r="I134" t="n">
-        <v>2</v>
+        <v>14</v>
       </c>
       <c r="J134" t="n">
         <v>10</v>
@@ -43972,10 +43972,10 @@
         <v>5</v>
       </c>
       <c r="T134" t="n">
+        <v>0</v>
+      </c>
+      <c r="U134" t="n">
         <v>1</v>
-      </c>
-      <c r="U134" t="n">
-        <v>0</v>
       </c>
       <c r="V134" t="n">
         <v>1</v>
@@ -44272,13 +44272,13 @@
         <v>12</v>
       </c>
       <c r="G137" t="n">
+        <v>4</v>
+      </c>
+      <c r="H137" t="n">
+        <v>6</v>
+      </c>
+      <c r="I137" t="n">
         <v>9</v>
-      </c>
-      <c r="H137" t="n">
-        <v>4</v>
-      </c>
-      <c r="I137" t="n">
-        <v>6</v>
       </c>
       <c r="J137" t="n">
         <v>27</v>
@@ -44311,10 +44311,10 @@
         <v>3</v>
       </c>
       <c r="T137" t="n">
+        <v>2</v>
+      </c>
+      <c r="U137" t="n">
         <v>1</v>
-      </c>
-      <c r="U137" t="n">
-        <v>2</v>
       </c>
       <c r="V137" t="n">
         <v>0</v>
@@ -44611,13 +44611,13 @@
         <v>8</v>
       </c>
       <c r="G140" t="n">
+        <v>0</v>
+      </c>
+      <c r="H140" t="n">
+        <v>5</v>
+      </c>
+      <c r="I140" t="n">
         <v>12</v>
-      </c>
-      <c r="H140" t="n">
-        <v>0</v>
-      </c>
-      <c r="I140" t="n">
-        <v>5</v>
       </c>
       <c r="J140" t="n">
         <v>6</v>
@@ -44650,10 +44650,10 @@
         <v>2</v>
       </c>
       <c r="T140" t="n">
+        <v>2</v>
+      </c>
+      <c r="U140" t="n">
         <v>1</v>
-      </c>
-      <c r="U140" t="n">
-        <v>2</v>
       </c>
       <c r="V140" t="n">
         <v>1</v>
@@ -44950,13 +44950,13 @@
         <v>8</v>
       </c>
       <c r="G143" t="n">
+        <v>1</v>
+      </c>
+      <c r="H143" t="n">
+        <v>15</v>
+      </c>
+      <c r="I143" t="n">
         <v>20</v>
-      </c>
-      <c r="H143" t="n">
-        <v>1</v>
-      </c>
-      <c r="I143" t="n">
-        <v>15</v>
       </c>
       <c r="J143" t="n">
         <v>23</v>
@@ -44989,10 +44989,10 @@
         <v>4</v>
       </c>
       <c r="T143" t="n">
+        <v>1</v>
+      </c>
+      <c r="U143" t="n">
         <v>3</v>
-      </c>
-      <c r="U143" t="n">
-        <v>1</v>
       </c>
       <c r="V143" t="n">
         <v>1</v>
@@ -45289,13 +45289,13 @@
         <v>16</v>
       </c>
       <c r="G146" t="n">
+        <v>2</v>
+      </c>
+      <c r="H146" t="n">
+        <v>8</v>
+      </c>
+      <c r="I146" t="n">
         <v>11</v>
-      </c>
-      <c r="H146" t="n">
-        <v>2</v>
-      </c>
-      <c r="I146" t="n">
-        <v>8</v>
       </c>
       <c r="J146" t="n">
         <v>14</v>
@@ -45328,10 +45328,10 @@
         <v>7</v>
       </c>
       <c r="T146" t="n">
+        <v>1</v>
+      </c>
+      <c r="U146" t="n">
         <v>2</v>
-      </c>
-      <c r="U146" t="n">
-        <v>1</v>
       </c>
       <c r="V146" t="n">
         <v>0</v>
@@ -45628,13 +45628,13 @@
         <v>3</v>
       </c>
       <c r="G149" t="n">
+        <v>1</v>
+      </c>
+      <c r="H149" t="n">
+        <v>7</v>
+      </c>
+      <c r="I149" t="n">
         <v>3</v>
-      </c>
-      <c r="H149" t="n">
-        <v>1</v>
-      </c>
-      <c r="I149" t="n">
-        <v>7</v>
       </c>
       <c r="J149" t="n">
         <v>9</v>
@@ -45667,10 +45667,10 @@
         <v>4</v>
       </c>
       <c r="T149" t="n">
+        <v>0</v>
+      </c>
+      <c r="U149" t="n">
         <v>2</v>
-      </c>
-      <c r="U149" t="n">
-        <v>0</v>
       </c>
       <c r="V149" t="n">
         <v>0</v>
@@ -45967,13 +45967,13 @@
         <v>9</v>
       </c>
       <c r="G152" t="n">
+        <v>1</v>
+      </c>
+      <c r="H152" t="n">
+        <v>4</v>
+      </c>
+      <c r="I152" t="n">
         <v>11</v>
-      </c>
-      <c r="H152" t="n">
-        <v>1</v>
-      </c>
-      <c r="I152" t="n">
-        <v>4</v>
       </c>
       <c r="J152" t="n">
         <v>8</v>
@@ -46006,10 +46006,10 @@
         <v>5</v>
       </c>
       <c r="T152" t="n">
+        <v>0</v>
+      </c>
+      <c r="U152" t="n">
         <v>4</v>
-      </c>
-      <c r="U152" t="n">
-        <v>0</v>
       </c>
       <c r="V152" t="n">
         <v>0</v>
@@ -46306,13 +46306,13 @@
         <v>4</v>
       </c>
       <c r="G155" t="n">
+        <v>0</v>
+      </c>
+      <c r="H155" t="n">
+        <v>4</v>
+      </c>
+      <c r="I155" t="n">
         <v>5</v>
-      </c>
-      <c r="H155" t="n">
-        <v>0</v>
-      </c>
-      <c r="I155" t="n">
-        <v>4</v>
       </c>
       <c r="J155" t="n">
         <v>8</v>
@@ -46345,10 +46345,10 @@
         <v>4</v>
       </c>
       <c r="T155" t="n">
+        <v>0</v>
+      </c>
+      <c r="U155" t="n">
         <v>1</v>
-      </c>
-      <c r="U155" t="n">
-        <v>0</v>
       </c>
       <c r="V155" t="n">
         <v>0</v>
@@ -46645,13 +46645,13 @@
         <v>7</v>
       </c>
       <c r="G158" t="n">
+        <v>0</v>
+      </c>
+      <c r="H158" t="n">
+        <v>4</v>
+      </c>
+      <c r="I158" t="n">
         <v>11</v>
-      </c>
-      <c r="H158" t="n">
-        <v>0</v>
-      </c>
-      <c r="I158" t="n">
-        <v>4</v>
       </c>
       <c r="J158" t="n">
         <v>14</v>
@@ -46684,10 +46684,10 @@
         <v>2</v>
       </c>
       <c r="T158" t="n">
+        <v>1</v>
+      </c>
+      <c r="U158" t="n">
         <v>2</v>
-      </c>
-      <c r="U158" t="n">
-        <v>1</v>
       </c>
       <c r="V158" t="n">
         <v>0</v>
@@ -46984,10 +46984,10 @@
         <v>11</v>
       </c>
       <c r="G161" t="n">
+        <v>0</v>
+      </c>
+      <c r="H161" t="n">
         <v>8</v>
-      </c>
-      <c r="H161" t="n">
-        <v>0</v>
       </c>
       <c r="I161" t="n">
         <v>8</v>
@@ -47023,10 +47023,10 @@
         <v>3</v>
       </c>
       <c r="T161" t="n">
+        <v>0</v>
+      </c>
+      <c r="U161" t="n">
         <v>1</v>
-      </c>
-      <c r="U161" t="n">
-        <v>0</v>
       </c>
       <c r="V161" t="n">
         <v>1</v>
@@ -47323,13 +47323,13 @@
         <v>14</v>
       </c>
       <c r="G164" t="n">
+        <v>0</v>
+      </c>
+      <c r="H164" t="n">
+        <v>7</v>
+      </c>
+      <c r="I164" t="n">
         <v>15</v>
-      </c>
-      <c r="H164" t="n">
-        <v>0</v>
-      </c>
-      <c r="I164" t="n">
-        <v>7</v>
       </c>
       <c r="J164" t="n">
         <v>24</v>
@@ -47362,10 +47362,10 @@
         <v>7</v>
       </c>
       <c r="T164" t="n">
+        <v>0</v>
+      </c>
+      <c r="U164" t="n">
         <v>2</v>
-      </c>
-      <c r="U164" t="n">
-        <v>0</v>
       </c>
       <c r="V164" t="n">
         <v>1</v>
@@ -47662,13 +47662,13 @@
         <v>10</v>
       </c>
       <c r="G167" t="n">
+        <v>0</v>
+      </c>
+      <c r="H167" t="n">
+        <v>11</v>
+      </c>
+      <c r="I167" t="n">
         <v>9</v>
-      </c>
-      <c r="H167" t="n">
-        <v>0</v>
-      </c>
-      <c r="I167" t="n">
-        <v>11</v>
       </c>
       <c r="J167" t="n">
         <v>14</v>
@@ -48001,13 +48001,13 @@
         <v>26</v>
       </c>
       <c r="G170" t="n">
+        <v>0</v>
+      </c>
+      <c r="H170" t="n">
+        <v>18</v>
+      </c>
+      <c r="I170" t="n">
         <v>13</v>
-      </c>
-      <c r="H170" t="n">
-        <v>0</v>
-      </c>
-      <c r="I170" t="n">
-        <v>18</v>
       </c>
       <c r="J170" t="n">
         <v>39</v>
@@ -48040,10 +48040,10 @@
         <v>6</v>
       </c>
       <c r="T170" t="n">
+        <v>0</v>
+      </c>
+      <c r="U170" t="n">
         <v>3</v>
-      </c>
-      <c r="U170" t="n">
-        <v>0</v>
       </c>
       <c r="V170" t="n">
         <v>0</v>
@@ -48340,13 +48340,13 @@
         <v>4</v>
       </c>
       <c r="G173" t="n">
+        <v>0</v>
+      </c>
+      <c r="H173" t="n">
+        <v>8</v>
+      </c>
+      <c r="I173" t="n">
         <v>7</v>
-      </c>
-      <c r="H173" t="n">
-        <v>0</v>
-      </c>
-      <c r="I173" t="n">
-        <v>8</v>
       </c>
       <c r="J173" t="n">
         <v>10</v>
@@ -48379,10 +48379,10 @@
         <v>0</v>
       </c>
       <c r="T173" t="n">
+        <v>0</v>
+      </c>
+      <c r="U173" t="n">
         <v>1</v>
-      </c>
-      <c r="U173" t="n">
-        <v>0</v>
       </c>
       <c r="V173" t="n">
         <v>0</v>
@@ -48679,13 +48679,13 @@
         <v>9</v>
       </c>
       <c r="G176" t="n">
+        <v>0</v>
+      </c>
+      <c r="H176" t="n">
+        <v>5</v>
+      </c>
+      <c r="I176" t="n">
         <v>19</v>
-      </c>
-      <c r="H176" t="n">
-        <v>0</v>
-      </c>
-      <c r="I176" t="n">
-        <v>5</v>
       </c>
       <c r="J176" t="n">
         <v>22</v>
@@ -48718,10 +48718,10 @@
         <v>6</v>
       </c>
       <c r="T176" t="n">
+        <v>0</v>
+      </c>
+      <c r="U176" t="n">
         <v>1</v>
-      </c>
-      <c r="U176" t="n">
-        <v>0</v>
       </c>
       <c r="V176" t="n">
         <v>2</v>
@@ -49018,13 +49018,13 @@
         <v>14</v>
       </c>
       <c r="G179" t="n">
+        <v>1</v>
+      </c>
+      <c r="H179" t="n">
+        <v>10</v>
+      </c>
+      <c r="I179" t="n">
         <v>6</v>
-      </c>
-      <c r="H179" t="n">
-        <v>1</v>
-      </c>
-      <c r="I179" t="n">
-        <v>10</v>
       </c>
       <c r="J179" t="n">
         <v>11</v>
@@ -49057,10 +49057,10 @@
         <v>2</v>
       </c>
       <c r="T179" t="n">
+        <v>2</v>
+      </c>
+      <c r="U179" t="n">
         <v>3</v>
-      </c>
-      <c r="U179" t="n">
-        <v>2</v>
       </c>
       <c r="V179" t="n">
         <v>1</v>
@@ -49357,13 +49357,13 @@
         <v>11</v>
       </c>
       <c r="G182" t="n">
+        <v>0</v>
+      </c>
+      <c r="H182" t="n">
+        <v>2</v>
+      </c>
+      <c r="I182" t="n">
         <v>8</v>
-      </c>
-      <c r="H182" t="n">
-        <v>0</v>
-      </c>
-      <c r="I182" t="n">
-        <v>2</v>
       </c>
       <c r="J182" t="n">
         <v>13</v>
@@ -49396,10 +49396,10 @@
         <v>5</v>
       </c>
       <c r="T182" t="n">
+        <v>2</v>
+      </c>
+      <c r="U182" t="n">
         <v>1</v>
-      </c>
-      <c r="U182" t="n">
-        <v>2</v>
       </c>
       <c r="V182" t="n">
         <v>0</v>
@@ -49696,13 +49696,13 @@
         <v>24</v>
       </c>
       <c r="G185" t="n">
+        <v>0</v>
+      </c>
+      <c r="H185" t="n">
+        <v>13</v>
+      </c>
+      <c r="I185" t="n">
         <v>17</v>
-      </c>
-      <c r="H185" t="n">
-        <v>0</v>
-      </c>
-      <c r="I185" t="n">
-        <v>13</v>
       </c>
       <c r="J185" t="n">
         <v>16</v>
@@ -49735,10 +49735,10 @@
         <v>6</v>
       </c>
       <c r="T185" t="n">
+        <v>2</v>
+      </c>
+      <c r="U185" t="n">
         <v>4</v>
-      </c>
-      <c r="U185" t="n">
-        <v>2</v>
       </c>
       <c r="V185" t="n">
         <v>0</v>
@@ -50035,10 +50035,10 @@
         <v>16</v>
       </c>
       <c r="G188" t="n">
+        <v>0</v>
+      </c>
+      <c r="H188" t="n">
         <v>9</v>
-      </c>
-      <c r="H188" t="n">
-        <v>0</v>
       </c>
       <c r="I188" t="n">
         <v>9</v>
@@ -50074,10 +50074,10 @@
         <v>4</v>
       </c>
       <c r="T188" t="n">
+        <v>0</v>
+      </c>
+      <c r="U188" t="n">
         <v>1</v>
-      </c>
-      <c r="U188" t="n">
-        <v>0</v>
       </c>
       <c r="V188" t="n">
         <v>0</v>
@@ -50374,13 +50374,13 @@
         <v>9</v>
       </c>
       <c r="G191" t="n">
+        <v>0</v>
+      </c>
+      <c r="H191" t="n">
+        <v>6</v>
+      </c>
+      <c r="I191" t="n">
         <v>9</v>
-      </c>
-      <c r="H191" t="n">
-        <v>0</v>
-      </c>
-      <c r="I191" t="n">
-        <v>6</v>
       </c>
       <c r="J191" t="n">
         <v>11</v>
@@ -50413,10 +50413,10 @@
         <v>2</v>
       </c>
       <c r="T191" t="n">
+        <v>1</v>
+      </c>
+      <c r="U191" t="n">
         <v>3</v>
-      </c>
-      <c r="U191" t="n">
-        <v>1</v>
       </c>
       <c r="V191" t="n">
         <v>0</v>
@@ -50713,13 +50713,13 @@
         <v>8</v>
       </c>
       <c r="G194" t="n">
+        <v>0</v>
+      </c>
+      <c r="H194" t="n">
+        <v>6</v>
+      </c>
+      <c r="I194" t="n">
         <v>16</v>
-      </c>
-      <c r="H194" t="n">
-        <v>0</v>
-      </c>
-      <c r="I194" t="n">
-        <v>6</v>
       </c>
       <c r="J194" t="n">
         <v>10</v>
@@ -50752,10 +50752,10 @@
         <v>4</v>
       </c>
       <c r="T194" t="n">
+        <v>0</v>
+      </c>
+      <c r="U194" t="n">
         <v>1</v>
-      </c>
-      <c r="U194" t="n">
-        <v>0</v>
       </c>
       <c r="V194" t="n">
         <v>0</v>
@@ -51052,13 +51052,13 @@
         <v>6</v>
       </c>
       <c r="G197" t="n">
+        <v>0</v>
+      </c>
+      <c r="H197" t="n">
+        <v>4</v>
+      </c>
+      <c r="I197" t="n">
         <v>7</v>
-      </c>
-      <c r="H197" t="n">
-        <v>0</v>
-      </c>
-      <c r="I197" t="n">
-        <v>4</v>
       </c>
       <c r="J197" t="n">
         <v>11</v>
@@ -51391,13 +51391,13 @@
         <v>13</v>
       </c>
       <c r="G200" t="n">
+        <v>0</v>
+      </c>
+      <c r="H200" t="n">
+        <v>7</v>
+      </c>
+      <c r="I200" t="n">
         <v>10</v>
-      </c>
-      <c r="H200" t="n">
-        <v>0</v>
-      </c>
-      <c r="I200" t="n">
-        <v>7</v>
       </c>
       <c r="J200" t="n">
         <v>13</v>
@@ -51730,13 +51730,13 @@
         <v>13</v>
       </c>
       <c r="G203" t="n">
+        <v>0</v>
+      </c>
+      <c r="H203" t="n">
+        <v>16</v>
+      </c>
+      <c r="I203" t="n">
         <v>10</v>
-      </c>
-      <c r="H203" t="n">
-        <v>0</v>
-      </c>
-      <c r="I203" t="n">
-        <v>16</v>
       </c>
       <c r="J203" t="n">
         <v>16</v>
@@ -51769,10 +51769,10 @@
         <v>7</v>
       </c>
       <c r="T203" t="n">
+        <v>4</v>
+      </c>
+      <c r="U203" t="n">
         <v>3</v>
-      </c>
-      <c r="U203" t="n">
-        <v>4</v>
       </c>
       <c r="V203" t="n">
         <v>0</v>
@@ -52069,13 +52069,13 @@
         <v>14</v>
       </c>
       <c r="G206" t="n">
+        <v>0</v>
+      </c>
+      <c r="H206" t="n">
+        <v>13</v>
+      </c>
+      <c r="I206" t="n">
         <v>12</v>
-      </c>
-      <c r="H206" t="n">
-        <v>0</v>
-      </c>
-      <c r="I206" t="n">
-        <v>13</v>
       </c>
       <c r="J206" t="n">
         <v>23</v>
@@ -52108,10 +52108,10 @@
         <v>3</v>
       </c>
       <c r="T206" t="n">
+        <v>0</v>
+      </c>
+      <c r="U206" t="n">
         <v>1</v>
-      </c>
-      <c r="U206" t="n">
-        <v>0</v>
       </c>
       <c r="V206" t="n">
         <v>0</v>
@@ -52408,13 +52408,13 @@
         <v>6</v>
       </c>
       <c r="G209" t="n">
+        <v>1</v>
+      </c>
+      <c r="H209" t="n">
+        <v>7</v>
+      </c>
+      <c r="I209" t="n">
         <v>10</v>
-      </c>
-      <c r="H209" t="n">
-        <v>1</v>
-      </c>
-      <c r="I209" t="n">
-        <v>7</v>
       </c>
       <c r="J209" t="n">
         <v>16</v>
@@ -52447,10 +52447,10 @@
         <v>2</v>
       </c>
       <c r="T209" t="n">
+        <v>0</v>
+      </c>
+      <c r="U209" t="n">
         <v>2</v>
-      </c>
-      <c r="U209" t="n">
-        <v>0</v>
       </c>
       <c r="V209" t="n">
         <v>0</v>
@@ -52747,13 +52747,13 @@
         <v>2</v>
       </c>
       <c r="G212" t="n">
+        <v>0</v>
+      </c>
+      <c r="H212" t="n">
+        <v>7</v>
+      </c>
+      <c r="I212" t="n">
         <v>6</v>
-      </c>
-      <c r="H212" t="n">
-        <v>0</v>
-      </c>
-      <c r="I212" t="n">
-        <v>7</v>
       </c>
       <c r="J212" t="n">
         <v>7</v>
@@ -52786,10 +52786,10 @@
         <v>1</v>
       </c>
       <c r="T212" t="n">
+        <v>0</v>
+      </c>
+      <c r="U212" t="n">
         <v>1</v>
-      </c>
-      <c r="U212" t="n">
-        <v>0</v>
       </c>
       <c r="V212" t="n">
         <v>0</v>
@@ -53086,13 +53086,13 @@
         <v>4</v>
       </c>
       <c r="G215" t="n">
+        <v>1</v>
+      </c>
+      <c r="H215" t="n">
+        <v>6</v>
+      </c>
+      <c r="I215" t="n">
         <v>14</v>
-      </c>
-      <c r="H215" t="n">
-        <v>1</v>
-      </c>
-      <c r="I215" t="n">
-        <v>6</v>
       </c>
       <c r="J215" t="n">
         <v>10</v>
@@ -53125,10 +53125,10 @@
         <v>5</v>
       </c>
       <c r="T215" t="n">
+        <v>3</v>
+      </c>
+      <c r="U215" t="n">
         <v>2</v>
-      </c>
-      <c r="U215" t="n">
-        <v>3</v>
       </c>
       <c r="V215" t="n">
         <v>1</v>
@@ -53425,13 +53425,13 @@
         <v>8</v>
       </c>
       <c r="G218" t="n">
+        <v>0</v>
+      </c>
+      <c r="H218" t="n">
+        <v>4</v>
+      </c>
+      <c r="I218" t="n">
         <v>14</v>
-      </c>
-      <c r="H218" t="n">
-        <v>0</v>
-      </c>
-      <c r="I218" t="n">
-        <v>4</v>
       </c>
       <c r="J218" t="n">
         <v>17</v>
@@ -53464,10 +53464,10 @@
         <v>4</v>
       </c>
       <c r="T218" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U218" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="V218" t="n">
         <v>0</v>
@@ -53764,13 +53764,13 @@
         <v>4</v>
       </c>
       <c r="G221" t="n">
+        <v>1</v>
+      </c>
+      <c r="H221" t="n">
+        <v>6</v>
+      </c>
+      <c r="I221" t="n">
         <v>14</v>
-      </c>
-      <c r="H221" t="n">
-        <v>1</v>
-      </c>
-      <c r="I221" t="n">
-        <v>6</v>
       </c>
       <c r="J221" t="n">
         <v>15</v>
@@ -53803,10 +53803,10 @@
         <v>1</v>
       </c>
       <c r="T221" t="n">
+        <v>2</v>
+      </c>
+      <c r="U221" t="n">
         <v>7</v>
-      </c>
-      <c r="U221" t="n">
-        <v>2</v>
       </c>
       <c r="V221" t="n">
         <v>0</v>
@@ -54103,13 +54103,13 @@
         <v>2</v>
       </c>
       <c r="G224" t="n">
+        <v>0</v>
+      </c>
+      <c r="H224" t="n">
+        <v>4</v>
+      </c>
+      <c r="I224" t="n">
         <v>15</v>
-      </c>
-      <c r="H224" t="n">
-        <v>0</v>
-      </c>
-      <c r="I224" t="n">
-        <v>4</v>
       </c>
       <c r="J224" t="n">
         <v>9</v>
@@ -54142,10 +54142,10 @@
         <v>1</v>
       </c>
       <c r="T224" t="n">
+        <v>1</v>
+      </c>
+      <c r="U224" t="n">
         <v>2</v>
-      </c>
-      <c r="U224" t="n">
-        <v>1</v>
       </c>
       <c r="V224" t="n">
         <v>0</v>
@@ -54442,13 +54442,13 @@
         <v>13</v>
       </c>
       <c r="G227" t="n">
+        <v>0</v>
+      </c>
+      <c r="H227" t="n">
+        <v>15</v>
+      </c>
+      <c r="I227" t="n">
         <v>12</v>
-      </c>
-      <c r="H227" t="n">
-        <v>0</v>
-      </c>
-      <c r="I227" t="n">
-        <v>15</v>
       </c>
       <c r="J227" t="n">
         <v>23</v>
@@ -54481,10 +54481,10 @@
         <v>4</v>
       </c>
       <c r="T227" t="n">
+        <v>1</v>
+      </c>
+      <c r="U227" t="n">
         <v>2</v>
-      </c>
-      <c r="U227" t="n">
-        <v>1</v>
       </c>
       <c r="V227" t="n">
         <v>0</v>
@@ -54781,13 +54781,13 @@
         <v>5</v>
       </c>
       <c r="G230" t="n">
+        <v>1</v>
+      </c>
+      <c r="H230" t="n">
+        <v>10</v>
+      </c>
+      <c r="I230" t="n">
         <v>9</v>
-      </c>
-      <c r="H230" t="n">
-        <v>1</v>
-      </c>
-      <c r="I230" t="n">
-        <v>10</v>
       </c>
       <c r="J230" t="n">
         <v>31</v>
@@ -54820,10 +54820,10 @@
         <v>6</v>
       </c>
       <c r="T230" t="n">
+        <v>1</v>
+      </c>
+      <c r="U230" t="n">
         <v>2</v>
-      </c>
-      <c r="U230" t="n">
-        <v>1</v>
       </c>
       <c r="V230" t="n">
         <v>0</v>
@@ -55120,13 +55120,13 @@
         <v>3</v>
       </c>
       <c r="G233" t="n">
+        <v>0</v>
+      </c>
+      <c r="H233" t="n">
+        <v>8</v>
+      </c>
+      <c r="I233" t="n">
         <v>5</v>
-      </c>
-      <c r="H233" t="n">
-        <v>0</v>
-      </c>
-      <c r="I233" t="n">
-        <v>8</v>
       </c>
       <c r="J233" t="n">
         <v>8</v>
@@ -55159,10 +55159,10 @@
         <v>5</v>
       </c>
       <c r="T233" t="n">
+        <v>1</v>
+      </c>
+      <c r="U233" t="n">
         <v>2</v>
-      </c>
-      <c r="U233" t="n">
-        <v>1</v>
       </c>
       <c r="V233" t="n">
         <v>0</v>
@@ -55459,13 +55459,13 @@
         <v>3</v>
       </c>
       <c r="G236" t="n">
+        <v>0</v>
+      </c>
+      <c r="H236" t="n">
+        <v>6</v>
+      </c>
+      <c r="I236" t="n">
         <v>9</v>
-      </c>
-      <c r="H236" t="n">
-        <v>0</v>
-      </c>
-      <c r="I236" t="n">
-        <v>6</v>
       </c>
       <c r="J236" t="n">
         <v>6</v>
@@ -55798,13 +55798,13 @@
         <v>19</v>
       </c>
       <c r="G239" t="n">
+        <v>1</v>
+      </c>
+      <c r="H239" t="n">
+        <v>7</v>
+      </c>
+      <c r="I239" t="n">
         <v>9</v>
-      </c>
-      <c r="H239" t="n">
-        <v>1</v>
-      </c>
-      <c r="I239" t="n">
-        <v>7</v>
       </c>
       <c r="J239" t="n">
         <v>21</v>
@@ -55837,10 +55837,10 @@
         <v>2</v>
       </c>
       <c r="T239" t="n">
+        <v>0</v>
+      </c>
+      <c r="U239" t="n">
         <v>2</v>
-      </c>
-      <c r="U239" t="n">
-        <v>0</v>
       </c>
       <c r="V239" t="n">
         <v>0</v>
@@ -56137,13 +56137,13 @@
         <v>12</v>
       </c>
       <c r="G242" t="n">
+        <v>0</v>
+      </c>
+      <c r="H242" t="n">
+        <v>7</v>
+      </c>
+      <c r="I242" t="n">
         <v>11</v>
-      </c>
-      <c r="H242" t="n">
-        <v>0</v>
-      </c>
-      <c r="I242" t="n">
-        <v>7</v>
       </c>
       <c r="J242" t="n">
         <v>17</v>
@@ -56176,10 +56176,10 @@
         <v>3</v>
       </c>
       <c r="T242" t="n">
+        <v>1</v>
+      </c>
+      <c r="U242" t="n">
         <v>2</v>
-      </c>
-      <c r="U242" t="n">
-        <v>1</v>
       </c>
       <c r="V242" t="n">
         <v>0</v>
@@ -56476,13 +56476,13 @@
         <v>9</v>
       </c>
       <c r="G245" t="n">
+        <v>1</v>
+      </c>
+      <c r="H245" t="n">
+        <v>10</v>
+      </c>
+      <c r="I245" t="n">
         <v>13</v>
-      </c>
-      <c r="H245" t="n">
-        <v>1</v>
-      </c>
-      <c r="I245" t="n">
-        <v>10</v>
       </c>
       <c r="J245" t="n">
         <v>27</v>
@@ -56515,10 +56515,10 @@
         <v>3</v>
       </c>
       <c r="T245" t="n">
+        <v>1</v>
+      </c>
+      <c r="U245" t="n">
         <v>2</v>
-      </c>
-      <c r="U245" t="n">
-        <v>1</v>
       </c>
       <c r="V245" t="n">
         <v>0</v>
@@ -56815,13 +56815,13 @@
         <v>16</v>
       </c>
       <c r="G248" t="n">
+        <v>0</v>
+      </c>
+      <c r="H248" t="n">
+        <v>7</v>
+      </c>
+      <c r="I248" t="n">
         <v>14</v>
-      </c>
-      <c r="H248" t="n">
-        <v>0</v>
-      </c>
-      <c r="I248" t="n">
-        <v>7</v>
       </c>
       <c r="J248" t="n">
         <v>7</v>
@@ -56854,10 +56854,10 @@
         <v>8</v>
       </c>
       <c r="T248" t="n">
+        <v>3</v>
+      </c>
+      <c r="U248" t="n">
         <v>1</v>
-      </c>
-      <c r="U248" t="n">
-        <v>3</v>
       </c>
       <c r="V248" t="n">
         <v>0</v>
@@ -57154,13 +57154,13 @@
         <v>10</v>
       </c>
       <c r="G251" t="n">
+        <v>0</v>
+      </c>
+      <c r="H251" t="n">
+        <v>7</v>
+      </c>
+      <c r="I251" t="n">
         <v>8</v>
-      </c>
-      <c r="H251" t="n">
-        <v>0</v>
-      </c>
-      <c r="I251" t="n">
-        <v>7</v>
       </c>
       <c r="J251" t="n">
         <v>12</v>
@@ -57193,10 +57193,10 @@
         <v>1</v>
       </c>
       <c r="T251" t="n">
+        <v>0</v>
+      </c>
+      <c r="U251" t="n">
         <v>4</v>
-      </c>
-      <c r="U251" t="n">
-        <v>0</v>
       </c>
       <c r="V251" t="n">
         <v>0</v>
@@ -57493,13 +57493,13 @@
         <v>6</v>
       </c>
       <c r="G254" t="n">
+        <v>0</v>
+      </c>
+      <c r="H254" t="n">
+        <v>5</v>
+      </c>
+      <c r="I254" t="n">
         <v>7</v>
-      </c>
-      <c r="H254" t="n">
-        <v>0</v>
-      </c>
-      <c r="I254" t="n">
-        <v>5</v>
       </c>
       <c r="J254" t="n">
         <v>18</v>
@@ -57532,10 +57532,10 @@
         <v>1</v>
       </c>
       <c r="T254" t="n">
+        <v>3</v>
+      </c>
+      <c r="U254" t="n">
         <v>4</v>
-      </c>
-      <c r="U254" t="n">
-        <v>3</v>
       </c>
       <c r="V254" t="n">
         <v>0</v>
@@ -57832,13 +57832,13 @@
         <v>11</v>
       </c>
       <c r="G257" t="n">
+        <v>1</v>
+      </c>
+      <c r="H257" t="n">
+        <v>7</v>
+      </c>
+      <c r="I257" t="n">
         <v>11</v>
-      </c>
-      <c r="H257" t="n">
-        <v>1</v>
-      </c>
-      <c r="I257" t="n">
-        <v>7</v>
       </c>
       <c r="J257" t="n">
         <v>18</v>
@@ -57871,10 +57871,10 @@
         <v>5</v>
       </c>
       <c r="T257" t="n">
+        <v>0</v>
+      </c>
+      <c r="U257" t="n">
         <v>2</v>
-      </c>
-      <c r="U257" t="n">
-        <v>0</v>
       </c>
       <c r="V257" t="n">
         <v>0</v>
@@ -58171,13 +58171,13 @@
         <v>9</v>
       </c>
       <c r="G260" t="n">
+        <v>0</v>
+      </c>
+      <c r="H260" t="n">
+        <v>7</v>
+      </c>
+      <c r="I260" t="n">
         <v>9</v>
-      </c>
-      <c r="H260" t="n">
-        <v>0</v>
-      </c>
-      <c r="I260" t="n">
-        <v>7</v>
       </c>
       <c r="J260" t="n">
         <v>22</v>
@@ -58210,10 +58210,10 @@
         <v>0</v>
       </c>
       <c r="T260" t="n">
+        <v>0</v>
+      </c>
+      <c r="U260" t="n">
         <v>3</v>
-      </c>
-      <c r="U260" t="n">
-        <v>0</v>
       </c>
       <c r="V260" t="n">
         <v>0</v>
@@ -58510,13 +58510,13 @@
         <v>8</v>
       </c>
       <c r="G263" t="n">
+        <v>0</v>
+      </c>
+      <c r="H263" t="n">
+        <v>3</v>
+      </c>
+      <c r="I263" t="n">
         <v>11</v>
-      </c>
-      <c r="H263" t="n">
-        <v>0</v>
-      </c>
-      <c r="I263" t="n">
-        <v>3</v>
       </c>
       <c r="J263" t="n">
         <v>12</v>
@@ -58549,10 +58549,10 @@
         <v>0</v>
       </c>
       <c r="T263" t="n">
+        <v>0</v>
+      </c>
+      <c r="U263" t="n">
         <v>2</v>
-      </c>
-      <c r="U263" t="n">
-        <v>0</v>
       </c>
       <c r="V263" t="n">
         <v>0</v>
@@ -58849,13 +58849,13 @@
         <v>12</v>
       </c>
       <c r="G266" t="n">
+        <v>0</v>
+      </c>
+      <c r="H266" t="n">
+        <v>4</v>
+      </c>
+      <c r="I266" t="n">
         <v>9</v>
-      </c>
-      <c r="H266" t="n">
-        <v>0</v>
-      </c>
-      <c r="I266" t="n">
-        <v>4</v>
       </c>
       <c r="J266" t="n">
         <v>8</v>
@@ -58888,10 +58888,10 @@
         <v>0</v>
       </c>
       <c r="T266" t="n">
+        <v>0</v>
+      </c>
+      <c r="U266" t="n">
         <v>1</v>
-      </c>
-      <c r="U266" t="n">
-        <v>0</v>
       </c>
       <c r="V266" t="n">
         <v>0</v>
@@ -59188,10 +59188,10 @@
         <v>11</v>
       </c>
       <c r="G269" t="n">
+        <v>1</v>
+      </c>
+      <c r="H269" t="n">
         <v>18</v>
-      </c>
-      <c r="H269" t="n">
-        <v>1</v>
       </c>
       <c r="I269" t="n">
         <v>18</v>
@@ -59227,10 +59227,10 @@
         <v>1</v>
       </c>
       <c r="T269" t="n">
+        <v>0</v>
+      </c>
+      <c r="U269" t="n">
         <v>3</v>
-      </c>
-      <c r="U269" t="n">
-        <v>0</v>
       </c>
       <c r="V269" t="n">
         <v>0</v>
@@ -59527,13 +59527,13 @@
         <v>9</v>
       </c>
       <c r="G272" t="n">
+        <v>0</v>
+      </c>
+      <c r="H272" t="n">
+        <v>9</v>
+      </c>
+      <c r="I272" t="n">
         <v>6</v>
-      </c>
-      <c r="H272" t="n">
-        <v>0</v>
-      </c>
-      <c r="I272" t="n">
-        <v>9</v>
       </c>
       <c r="J272" t="n">
         <v>24</v>
@@ -59566,10 +59566,10 @@
         <v>0</v>
       </c>
       <c r="T272" t="n">
+        <v>0</v>
+      </c>
+      <c r="U272" t="n">
         <v>1</v>
-      </c>
-      <c r="U272" t="n">
-        <v>0</v>
       </c>
       <c r="V272" t="n">
         <v>0</v>
@@ -59866,13 +59866,13 @@
         <v>18</v>
       </c>
       <c r="G275" t="n">
+        <v>0</v>
+      </c>
+      <c r="H275" t="n">
+        <v>8</v>
+      </c>
+      <c r="I275" t="n">
         <v>6</v>
-      </c>
-      <c r="H275" t="n">
-        <v>0</v>
-      </c>
-      <c r="I275" t="n">
-        <v>8</v>
       </c>
       <c r="J275" t="n">
         <v>20</v>
@@ -59905,10 +59905,10 @@
         <v>0</v>
       </c>
       <c r="T275" t="n">
+        <v>0</v>
+      </c>
+      <c r="U275" t="n">
         <v>1</v>
-      </c>
-      <c r="U275" t="n">
-        <v>0</v>
       </c>
       <c r="V275" t="n">
         <v>0</v>
@@ -60205,13 +60205,13 @@
         <v>7</v>
       </c>
       <c r="G278" t="n">
+        <v>0</v>
+      </c>
+      <c r="H278" t="n">
+        <v>4</v>
+      </c>
+      <c r="I278" t="n">
         <v>7</v>
-      </c>
-      <c r="H278" t="n">
-        <v>0</v>
-      </c>
-      <c r="I278" t="n">
-        <v>4</v>
       </c>
       <c r="J278" t="n">
         <v>16</v>
@@ -60544,13 +60544,13 @@
         <v>10</v>
       </c>
       <c r="G281" t="n">
+        <v>0</v>
+      </c>
+      <c r="H281" t="n">
+        <v>12</v>
+      </c>
+      <c r="I281" t="n">
         <v>11</v>
-      </c>
-      <c r="H281" t="n">
-        <v>0</v>
-      </c>
-      <c r="I281" t="n">
-        <v>12</v>
       </c>
       <c r="J281" t="n">
         <v>31</v>
@@ -60583,10 +60583,10 @@
         <v>0</v>
       </c>
       <c r="T281" t="n">
+        <v>0</v>
+      </c>
+      <c r="U281" t="n">
         <v>3</v>
-      </c>
-      <c r="U281" t="n">
-        <v>0</v>
       </c>
       <c r="V281" t="n">
         <v>0</v>
@@ -60883,13 +60883,13 @@
         <v>12</v>
       </c>
       <c r="G284" t="n">
+        <v>0</v>
+      </c>
+      <c r="H284" t="n">
+        <v>8</v>
+      </c>
+      <c r="I284" t="n">
         <v>9</v>
-      </c>
-      <c r="H284" t="n">
-        <v>0</v>
-      </c>
-      <c r="I284" t="n">
-        <v>8</v>
       </c>
       <c r="J284" t="n">
         <v>4</v>
@@ -61222,13 +61222,13 @@
         <v>12</v>
       </c>
       <c r="G287" t="n">
+        <v>0</v>
+      </c>
+      <c r="H287" t="n">
+        <v>7</v>
+      </c>
+      <c r="I287" t="n">
         <v>2</v>
-      </c>
-      <c r="H287" t="n">
-        <v>0</v>
-      </c>
-      <c r="I287" t="n">
-        <v>7</v>
       </c>
       <c r="J287" t="n">
         <v>20</v>
@@ -61561,13 +61561,13 @@
         <v>10</v>
       </c>
       <c r="G290" t="n">
+        <v>0</v>
+      </c>
+      <c r="H290" t="n">
+        <v>12</v>
+      </c>
+      <c r="I290" t="n">
         <v>11</v>
-      </c>
-      <c r="H290" t="n">
-        <v>0</v>
-      </c>
-      <c r="I290" t="n">
-        <v>12</v>
       </c>
       <c r="J290" t="n">
         <v>12</v>
@@ -61600,10 +61600,10 @@
         <v>0</v>
       </c>
       <c r="T290" t="n">
+        <v>0</v>
+      </c>
+      <c r="U290" t="n">
         <v>3</v>
-      </c>
-      <c r="U290" t="n">
-        <v>0</v>
       </c>
       <c r="V290" t="n">
         <v>0</v>
@@ -61900,13 +61900,13 @@
         <v>8</v>
       </c>
       <c r="G293" t="n">
+        <v>0</v>
+      </c>
+      <c r="H293" t="n">
+        <v>1</v>
+      </c>
+      <c r="I293" t="n">
         <v>7</v>
-      </c>
-      <c r="H293" t="n">
-        <v>0</v>
-      </c>
-      <c r="I293" t="n">
-        <v>1</v>
       </c>
       <c r="J293" t="n">
         <v>15</v>
@@ -61939,10 +61939,10 @@
         <v>0</v>
       </c>
       <c r="T293" t="n">
+        <v>0</v>
+      </c>
+      <c r="U293" t="n">
         <v>2</v>
-      </c>
-      <c r="U293" t="n">
-        <v>0</v>
       </c>
       <c r="V293" t="n">
         <v>0</v>
@@ -62239,13 +62239,13 @@
         <v>7</v>
       </c>
       <c r="G296" t="n">
+        <v>0</v>
+      </c>
+      <c r="H296" t="n">
+        <v>4</v>
+      </c>
+      <c r="I296" t="n">
         <v>5</v>
-      </c>
-      <c r="H296" t="n">
-        <v>0</v>
-      </c>
-      <c r="I296" t="n">
-        <v>4</v>
       </c>
       <c r="J296" t="n">
         <v>11</v>
@@ -62278,10 +62278,10 @@
         <v>0</v>
       </c>
       <c r="T296" t="n">
+        <v>0</v>
+      </c>
+      <c r="U296" t="n">
         <v>3</v>
-      </c>
-      <c r="U296" t="n">
-        <v>0</v>
       </c>
       <c r="V296" t="n">
         <v>0</v>
@@ -62578,13 +62578,13 @@
         <v>5</v>
       </c>
       <c r="G299" t="n">
+        <v>0</v>
+      </c>
+      <c r="H299" t="n">
+        <v>10</v>
+      </c>
+      <c r="I299" t="n">
         <v>11</v>
-      </c>
-      <c r="H299" t="n">
-        <v>0</v>
-      </c>
-      <c r="I299" t="n">
-        <v>10</v>
       </c>
       <c r="J299" t="n">
         <v>18</v>
@@ -62617,10 +62617,10 @@
         <v>0</v>
       </c>
       <c r="T299" t="n">
+        <v>0</v>
+      </c>
+      <c r="U299" t="n">
         <v>1</v>
-      </c>
-      <c r="U299" t="n">
-        <v>0</v>
       </c>
       <c r="V299" t="n">
         <v>0</v>
@@ -62917,13 +62917,13 @@
         <v>17</v>
       </c>
       <c r="G302" t="n">
+        <v>0</v>
+      </c>
+      <c r="H302" t="n">
+        <v>12</v>
+      </c>
+      <c r="I302" t="n">
         <v>13</v>
-      </c>
-      <c r="H302" t="n">
-        <v>0</v>
-      </c>
-      <c r="I302" t="n">
-        <v>12</v>
       </c>
       <c r="J302" t="n">
         <v>26</v>
@@ -62956,10 +62956,10 @@
         <v>0</v>
       </c>
       <c r="T302" t="n">
+        <v>0</v>
+      </c>
+      <c r="U302" t="n">
         <v>2</v>
-      </c>
-      <c r="U302" t="n">
-        <v>0</v>
       </c>
       <c r="V302" t="n">
         <v>0</v>
@@ -63256,13 +63256,13 @@
         <v>8</v>
       </c>
       <c r="G305" t="n">
+        <v>0</v>
+      </c>
+      <c r="H305" t="n">
+        <v>7</v>
+      </c>
+      <c r="I305" t="n">
         <v>11</v>
-      </c>
-      <c r="H305" t="n">
-        <v>0</v>
-      </c>
-      <c r="I305" t="n">
-        <v>7</v>
       </c>
       <c r="J305" t="n">
         <v>25</v>
@@ -63295,10 +63295,10 @@
         <v>0</v>
       </c>
       <c r="T305" t="n">
+        <v>0</v>
+      </c>
+      <c r="U305" t="n">
         <v>2</v>
-      </c>
-      <c r="U305" t="n">
-        <v>0</v>
       </c>
       <c r="V305" t="n">
         <v>0</v>
@@ -63595,13 +63595,13 @@
         <v>12</v>
       </c>
       <c r="G308" t="n">
+        <v>0</v>
+      </c>
+      <c r="H308" t="n">
+        <v>2</v>
+      </c>
+      <c r="I308" t="n">
         <v>8</v>
-      </c>
-      <c r="H308" t="n">
-        <v>0</v>
-      </c>
-      <c r="I308" t="n">
-        <v>2</v>
       </c>
       <c r="J308" t="n">
         <v>22</v>
@@ -63934,13 +63934,13 @@
         <v>16</v>
       </c>
       <c r="G311" t="n">
+        <v>0</v>
+      </c>
+      <c r="H311" t="n">
+        <v>14</v>
+      </c>
+      <c r="I311" t="n">
         <v>23</v>
-      </c>
-      <c r="H311" t="n">
-        <v>0</v>
-      </c>
-      <c r="I311" t="n">
-        <v>14</v>
       </c>
       <c r="J311" t="n">
         <v>26</v>
@@ -63973,10 +63973,10 @@
         <v>0</v>
       </c>
       <c r="T311" t="n">
+        <v>0</v>
+      </c>
+      <c r="U311" t="n">
         <v>1</v>
-      </c>
-      <c r="U311" t="n">
-        <v>0</v>
       </c>
       <c r="V311" t="n">
         <v>0</v>
@@ -64273,13 +64273,13 @@
         <v>15</v>
       </c>
       <c r="G314" t="n">
+        <v>0</v>
+      </c>
+      <c r="H314" t="n">
+        <v>13</v>
+      </c>
+      <c r="I314" t="n">
         <v>8</v>
-      </c>
-      <c r="H314" t="n">
-        <v>0</v>
-      </c>
-      <c r="I314" t="n">
-        <v>13</v>
       </c>
       <c r="J314" t="n">
         <v>23</v>
@@ -64312,10 +64312,10 @@
         <v>0</v>
       </c>
       <c r="T314" t="n">
+        <v>0</v>
+      </c>
+      <c r="U314" t="n">
         <v>2</v>
-      </c>
-      <c r="U314" t="n">
-        <v>0</v>
       </c>
       <c r="V314" t="n">
         <v>0</v>
@@ -64612,13 +64612,13 @@
         <v>7</v>
       </c>
       <c r="G317" t="n">
+        <v>0</v>
+      </c>
+      <c r="H317" t="n">
+        <v>4</v>
+      </c>
+      <c r="I317" t="n">
         <v>9</v>
-      </c>
-      <c r="H317" t="n">
-        <v>0</v>
-      </c>
-      <c r="I317" t="n">
-        <v>4</v>
       </c>
       <c r="J317" t="n">
         <v>14</v>
@@ -64651,10 +64651,10 @@
         <v>0</v>
       </c>
       <c r="T317" t="n">
+        <v>0</v>
+      </c>
+      <c r="U317" t="n">
         <v>5</v>
-      </c>
-      <c r="U317" t="n">
-        <v>0</v>
       </c>
       <c r="V317" t="n">
         <v>0</v>
@@ -64951,13 +64951,13 @@
         <v>7</v>
       </c>
       <c r="G320" t="n">
+        <v>0</v>
+      </c>
+      <c r="H320" t="n">
+        <v>8</v>
+      </c>
+      <c r="I320" t="n">
         <v>11</v>
-      </c>
-      <c r="H320" t="n">
-        <v>0</v>
-      </c>
-      <c r="I320" t="n">
-        <v>8</v>
       </c>
       <c r="J320" t="n">
         <v>18</v>
@@ -64990,10 +64990,10 @@
         <v>0</v>
       </c>
       <c r="T320" t="n">
+        <v>0</v>
+      </c>
+      <c r="U320" t="n">
         <v>1</v>
-      </c>
-      <c r="U320" t="n">
-        <v>0</v>
       </c>
       <c r="V320" t="n">
         <v>0</v>
@@ -65290,13 +65290,13 @@
         <v>14</v>
       </c>
       <c r="G323" t="n">
+        <v>0</v>
+      </c>
+      <c r="H323" t="n">
+        <v>6</v>
+      </c>
+      <c r="I323" t="n">
         <v>7</v>
-      </c>
-      <c r="H323" t="n">
-        <v>0</v>
-      </c>
-      <c r="I323" t="n">
-        <v>6</v>
       </c>
       <c r="J323" t="n">
         <v>23</v>
@@ -65329,10 +65329,10 @@
         <v>0</v>
       </c>
       <c r="T323" t="n">
+        <v>0</v>
+      </c>
+      <c r="U323" t="n">
         <v>3</v>
-      </c>
-      <c r="U323" t="n">
-        <v>0</v>
       </c>
       <c r="V323" t="n">
         <v>0</v>
@@ -65629,13 +65629,13 @@
         <v>15</v>
       </c>
       <c r="G326" t="n">
+        <v>0</v>
+      </c>
+      <c r="H326" t="n">
+        <v>12</v>
+      </c>
+      <c r="I326" t="n">
         <v>10</v>
-      </c>
-      <c r="H326" t="n">
-        <v>0</v>
-      </c>
-      <c r="I326" t="n">
-        <v>12</v>
       </c>
       <c r="J326" t="n">
         <v>21</v>
@@ -65668,10 +65668,10 @@
         <v>0</v>
       </c>
       <c r="T326" t="n">
+        <v>0</v>
+      </c>
+      <c r="U326" t="n">
         <v>4</v>
-      </c>
-      <c r="U326" t="n">
-        <v>0</v>
       </c>
       <c r="V326" t="n">
         <v>0</v>
@@ -65968,13 +65968,13 @@
         <v>15</v>
       </c>
       <c r="G329" t="n">
+        <v>0</v>
+      </c>
+      <c r="H329" t="n">
+        <v>7</v>
+      </c>
+      <c r="I329" t="n">
         <v>6</v>
-      </c>
-      <c r="H329" t="n">
-        <v>0</v>
-      </c>
-      <c r="I329" t="n">
-        <v>7</v>
       </c>
       <c r="J329" t="n">
         <v>11</v>
@@ -66007,10 +66007,10 @@
         <v>0</v>
       </c>
       <c r="T329" t="n">
+        <v>0</v>
+      </c>
+      <c r="U329" t="n">
         <v>1</v>
-      </c>
-      <c r="U329" t="n">
-        <v>0</v>
       </c>
       <c r="V329" t="n">
         <v>0</v>
@@ -66307,13 +66307,13 @@
         <v>16</v>
       </c>
       <c r="G332" t="n">
+        <v>0</v>
+      </c>
+      <c r="H332" t="n">
+        <v>7</v>
+      </c>
+      <c r="I332" t="n">
         <v>13</v>
-      </c>
-      <c r="H332" t="n">
-        <v>0</v>
-      </c>
-      <c r="I332" t="n">
-        <v>7</v>
       </c>
       <c r="J332" t="n">
         <v>14</v>
@@ -66346,10 +66346,10 @@
         <v>0</v>
       </c>
       <c r="T332" t="n">
+        <v>0</v>
+      </c>
+      <c r="U332" t="n">
         <v>1</v>
-      </c>
-      <c r="U332" t="n">
-        <v>0</v>
       </c>
       <c r="V332" t="n">
         <v>0</v>
@@ -66646,13 +66646,13 @@
         <v>13</v>
       </c>
       <c r="G335" t="n">
+        <v>0</v>
+      </c>
+      <c r="H335" t="n">
+        <v>10</v>
+      </c>
+      <c r="I335" t="n">
         <v>12</v>
-      </c>
-      <c r="H335" t="n">
-        <v>0</v>
-      </c>
-      <c r="I335" t="n">
-        <v>10</v>
       </c>
       <c r="J335" t="n">
         <v>19</v>
@@ -66685,10 +66685,10 @@
         <v>0</v>
       </c>
       <c r="T335" t="n">
+        <v>0</v>
+      </c>
+      <c r="U335" t="n">
         <v>1</v>
-      </c>
-      <c r="U335" t="n">
-        <v>0</v>
       </c>
       <c r="V335" t="n">
         <v>0</v>
@@ -66985,13 +66985,13 @@
         <v>15</v>
       </c>
       <c r="G338" t="n">
+        <v>0</v>
+      </c>
+      <c r="H338" t="n">
+        <v>6</v>
+      </c>
+      <c r="I338" t="n">
         <v>9</v>
-      </c>
-      <c r="H338" t="n">
-        <v>0</v>
-      </c>
-      <c r="I338" t="n">
-        <v>6</v>
       </c>
       <c r="J338" t="n">
         <v>23</v>
@@ -67024,10 +67024,10 @@
         <v>0</v>
       </c>
       <c r="T338" t="n">
+        <v>0</v>
+      </c>
+      <c r="U338" t="n">
         <v>1</v>
-      </c>
-      <c r="U338" t="n">
-        <v>0</v>
       </c>
       <c r="V338" t="n">
         <v>0</v>
@@ -67324,13 +67324,13 @@
         <v>3</v>
       </c>
       <c r="G341" t="n">
+        <v>0</v>
+      </c>
+      <c r="H341" t="n">
+        <v>7</v>
+      </c>
+      <c r="I341" t="n">
         <v>10</v>
-      </c>
-      <c r="H341" t="n">
-        <v>0</v>
-      </c>
-      <c r="I341" t="n">
-        <v>7</v>
       </c>
       <c r="J341" t="n">
         <v>18</v>
@@ -67663,13 +67663,13 @@
         <v>14</v>
       </c>
       <c r="G344" t="n">
+        <v>0</v>
+      </c>
+      <c r="H344" t="n">
+        <v>13</v>
+      </c>
+      <c r="I344" t="n">
         <v>12</v>
-      </c>
-      <c r="H344" t="n">
-        <v>0</v>
-      </c>
-      <c r="I344" t="n">
-        <v>13</v>
       </c>
       <c r="J344" t="n">
         <v>14</v>
@@ -69084,93 +69084,93 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Tofu</t>
+          <t>Water</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>7449</v>
+        <v>3</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Forecasted</t>
+          <t>Par level</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>+5.00%</t>
+          <t>+30.32%</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>+9.54%</t>
+          <t>+33.33%</t>
         </is>
       </c>
       <c r="F17" t="n">
-        <v>1064.14</v>
+        <v>0.35</v>
       </c>
       <c r="G17" t="n">
-        <v>1064.14</v>
+        <v>0.35</v>
       </c>
       <c r="H17" t="n">
-        <v>709.4299999999999</v>
+        <v>0.23</v>
       </c>
       <c r="I17" t="n">
-        <v>1418.85</v>
+        <v>0.46</v>
       </c>
       <c r="J17" t="n">
-        <v>1418.85</v>
+        <v>0.46</v>
       </c>
       <c r="K17" t="n">
-        <v>1064.14</v>
+        <v>0.35</v>
       </c>
       <c r="L17" t="n">
-        <v>709.4299999999999</v>
+        <v>0.23</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Water</t>
+          <t>Tofu</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>3</v>
+        <v>7449</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Par level</t>
+          <t>Forecasted</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>+30.32%</t>
+          <t>+5.00%</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>+33.33%</t>
+          <t>+9.54%</t>
         </is>
       </c>
       <c r="F18" t="n">
-        <v>0.35</v>
+        <v>1064.14</v>
       </c>
       <c r="G18" t="n">
-        <v>0.35</v>
+        <v>1064.14</v>
       </c>
       <c r="H18" t="n">
-        <v>0.23</v>
+        <v>709.4299999999999</v>
       </c>
       <c r="I18" t="n">
-        <v>0.46</v>
+        <v>1418.85</v>
       </c>
       <c r="J18" t="n">
-        <v>0.46</v>
+        <v>1418.85</v>
       </c>
       <c r="K18" t="n">
-        <v>0.35</v>
+        <v>1064.14</v>
       </c>
       <c r="L18" t="n">
-        <v>0.23</v>
+        <v>709.4299999999999</v>
       </c>
     </row>
     <row r="19">

</xml_diff>